<commit_message>
31 testcases are executed
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>ADMIN@123</t>
+  </si>
+  <si>
+    <t>admin</t>
   </si>
   <si>
     <t>Admin123</t>
@@ -601,10 +604,10 @@
     </row>
     <row r="12" ht="17.4">
       <c r="A12" s="2" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -620,7 +623,7 @@
         <v>2</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -633,10 +636,10 @@
     </row>
     <row r="14" ht="17.4">
       <c r="A14" s="2" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -648,12 +651,7 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" ht="17.4">
-      <c r="A15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -821,7 +819,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>

</xml_diff>